<commit_message>
Added method-level RBAC for approvals and NLP actions
</commit_message>
<xml_diff>
--- a/excel_reports/DBA_Monthly_Report_2026_06.xlsx
+++ b/excel_reports/DBA_Monthly_Report_2026_06.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -526,6 +526,48 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -708,7 +750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -4451,6 +4493,96 @@
         </is>
       </c>
       <c r="I31" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-22 16:10:55</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>INC-0031</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DBA Monitoring</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+SQL Monitoring Summary
+Monitoring Time: 2026-06-22 16:10:53.154043
+Database: AdventureWorks2019
+CPU Monitoring:
+Session ID: 65
+Status: running
+CPU Time: 0
+Elapsed Time: 0
+Reads: 0
+Writes: 0
+Logical Reads: 0
+Alert: CPU Usage Within Normal Range
+--------------------------
+Session ID: 64
+Status: sleeping
+CPU Time: 0
+Elapsed Time: 0
+Reads: 0
+Writes: 0
+Logical Reads: 508
+Alert: CPU Usage Within Normal Range
+--------------------------
+Session ID: 63
+Status: sleeping
+CPU Time: 0
+Elapsed Time: 0
+Reads: 0
+Writes: 0
+Logical Reads: 102
+Alert: CPU Usage Within Normal Range
+--------------------------
+Session ID: 55
+Status: sleeping
+CPU Time: 0
+Elapsed Time: 0
+Reads: 0
+Writes: 0
+Logical Reads: 2648
+Alert: CPU Usage Within Normal Range
+--------------------------
+No blocking sessions detected.
+No long running queries detected.
+Overall Status: HEALTHY</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
         </is>
@@ -5884,7 +6016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -6759,6 +6891,38 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-22 16:10:55</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MONITORING_STARTED_FROM_UI</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SQL Server Monitoring Workflow</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Monitoring workflow started from FastAPI Monitoring UI.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6770,7 +6934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -7604,6 +7768,26 @@
       </c>
       <c r="F30" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-22 16:10:55</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>DBA Recommendation</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalize all  validation andworking on  documentation
</commit_message>
<xml_diff>
--- a/excel_reports/DBA_Monthly_Report_2026_06.xlsx
+++ b/excel_reports/DBA_Monthly_Report_2026_06.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -570,6 +570,48 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -750,7 +792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -4583,6 +4625,267 @@
         </is>
       </c>
       <c r="I32" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:03:49</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>INC-0032</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DBA Monitoring</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+SQL Monitoring Summary
+Monitoring Time: 2026-06-23 12:03:44.668018
+Database: AdventureWorks2019
+CPU Monitoring:
+Session ID: 52
+Status: running
+CPU Time: 18
+Elapsed Time: 18
+Reads: 0
+Writes: 0
+Logical Reads: 257
+Alert: CPU Usage Within Normal Range
+--------------------------
+No blocking sessions detected.
+No long running queries detected.
+Overall Status: HEALTHY</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:51</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>INC-0033</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DBA Monitoring</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+SQL Monitoring Summary
+Monitoring Time: 2026-06-26 10:10:46.477058
+Database: AdventureWorks2019
+CPU Monitoring:
+Session ID: 55
+Status: running
+CPU Time: 129
+Elapsed Time: 129
+Reads: 0
+Writes: 0
+Logical Reads: 20
+Alert: CPU Usage Within Normal Range
+--------------------------
+No blocking sessions detected.
+No long running queries detected.
+Overall Status: HEALTHY</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:56</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>INC-0034</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DBA Monitoring</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+SQL Monitoring Summary
+Monitoring Time: 2026-06-26 10:10:45.516022
+Database: AdventureWorks2019
+CPU Monitoring:
+Session ID: 52
+Status: running
+CPU Time: 214
+Elapsed Time: 215
+Reads: 0
+Writes: 0
+Logical Reads: 20
+Alert: CPU Usage Within Normal Range
+--------------------------
+No blocking sessions detected.
+No long running queries detected.
+Overall Status: HEALTHY</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:56</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>INC-0035</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DBA Monitoring</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+SQL Monitoring Summary
+Monitoring Time: 2026-06-26 10:10:44.953676
+Database: AdventureWorks2019
+CPU Monitoring:
+Session ID: 54
+Status: running
+CPU Time: 20
+Elapsed Time: 20
+Reads: 0
+Writes: 0
+Logical Reads: 257
+Alert: CPU Usage Within Normal Range
+--------------------------
+Session ID: 52
+Status: running
+CPU Time: 20
+Elapsed Time: 20
+Reads: 0
+Writes: 0
+Logical Reads: 0
+Alert: CPU Usage Within Normal Range
+--------------------------
+No blocking sessions detected.
+No long running queries detected.
+Overall Status: HEALTHY</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
         <is>
           <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
         </is>
@@ -4880,7 +5183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5549,6 +5852,174 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16983979-efcc-4dbc-b7de-12f1bb34271f</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-18 15:38:38</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>NLP DBA Assistant</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FULL_DATABASE_BACKUP</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:04:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>57a88ccd-7337-424f-8897-891fcf2148b2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-18 15:48:48</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>NLP DBA Assistant</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FULL_DATABASE_BACKUP</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:34:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>c6583d38-9408-410b-8773-a5c5bf14b060</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:53:42</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NLP DBA Assistant</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>FULL_DATABASE_BACKUP</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:39:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>07b2b058-3e77-4ff0-89c9-572d4010c748</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-18 15:49:47</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NLP DBA Assistant</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FULL_DATABASE_BACKUP</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:11:10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5560,7 +6031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -6005,6 +6476,105 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EXEC-20260623120424003940</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:04:24</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FULL_DATABASE_BACKUP</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>AdventureWorks2019</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED_ACTION</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No execution handler found for this approved action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EXEC-20260623153438096512</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:34:38</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>RESTART_SQL_AGENT_JOB</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>syspolicy_purge_history</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>RUNBOOK_REQUEST_CREATED</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Azure Automation runbook request created after approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EXEC-20260626101119939464</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:11:19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>RESTART_SQL_AGENT_JOB</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>syspolicy_purge_history</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>RUNBOOK_REQUEST_CREATED</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Azure Automation runbook request created after approval.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6016,12 +6586,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
@@ -6920,6 +7490,326 @@
       <c r="F28" t="inlineStr">
         <is>
           <t>Monitoring workflow started from FastAPI Monitoring UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:04:17</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>APPROVAL_APPROVED</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Governance Approval</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Approval request approved from FastAPI Governance dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:04:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>REMEDIATION_EXECUTION_UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>AdventureWorks2019</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED_ACTION</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>No execution handler found for this approved action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:34:32</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>APPROVAL_APPROVED</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Governance Approval</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Approval request approved from FastAPI Governance dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:34:38</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>REMEDIATION_EXECUTED</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>syspolicy_purge_history</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>RUNBOOK_REQUEST_CREATED</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Approved remediation execution completed in simulated mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:39:14</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>APPROVAL_REJECTED</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Governance Approval</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Approval request rejected from FastAPI Governance dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:51</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MONITORING_STARTED_FROM_UI</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SQL Server Monitoring Workflow</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Monitoring workflow started from FastAPI Monitoring UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:56</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MONITORING_STARTED_FROM_UI</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SQL Server Monitoring Workflow</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Monitoring workflow started from FastAPI Monitoring UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:57</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MONITORING_STARTED_FROM_UI</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SQL Server Monitoring Workflow</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Monitoring workflow started from FastAPI Monitoring UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:11:10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>APPROVAL_APPROVED</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Governance Approval</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Approval request approved from FastAPI Governance dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:11:19</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Lead DBA</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>REMEDIATION_EXECUTED</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>syspolicy_purge_history</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>RUNBOOK_REQUEST_CREATED</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Approved remediation execution completed in simulated mode.</t>
         </is>
       </c>
     </row>
@@ -6934,7 +7824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -7788,6 +8678,66 @@
       </c>
       <c r="F31" t="inlineStr"/>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:03:49</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>DBA Recommendation</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:51</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>DBA Recommendation</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-26 10:10:56</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>DBA Recommendation</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>{"summary": "\n\nSystem Health Summary:\nMonitoring completed successfully for the SQL Server environment.\n\nMonitoring Observations:\n- CPU usage was captured successfully.\n- Blocking and long-running query checks were performed.\n- Database size information was retrieved successfully.\n\nRecommended Actions:\n- Continue regular monitoring.\n- Review workload trends periodically.\n- Maintain index and statistics upkeep.\n\nPrevention Recommendations:\n- Keep alert thresholds in place.\n- Perform routine capacity planning.\n- Maintain documentation and operational logs.\n\n", "root_cause": "AI analysis response was not structured.", "recommendation": "Continue monitoring and review SQL health manually.", "severity": "LOW"}</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>